<commit_message>
multiple regressions for final results in hysteresis paper
</commit_message>
<xml_diff>
--- a/correlations/multiple_regressions/multiple_regressions_summer.xlsx
+++ b/correlations/multiple_regressions/multiple_regressions_summer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\hysteresis\correlations\multiple_regressions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E312A13F-57E1-4651-910C-C4EF7B13CC8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A96D7395-9DBD-4AA5-A198-15B45DAF3C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E38EDDB9-EDBE-4091-BB71-D763E20009C1}"/>
+    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{E38EDDB9-EDBE-4091-BB71-D763E20009C1}"/>
   </bookViews>
   <sheets>
     <sheet name="summer" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="88">
   <si>
     <t>SSC (mg/L)</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>tauc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downstream </t>
   </si>
 </sst>
 </file>
@@ -866,6 +869,16 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -901,16 +914,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4038,7 +4041,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Aich HI to Excess Balance</a:t>
+              <a:t>Aich HI SSC to Excess Balance</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -4179,10 +4182,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>summer!$X$26:$X$36</c:f>
+              <c:f>summer!$X$26:$X$32</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>8.8732929175135894E-2</c:v>
                 </c:pt>
@@ -4204,18 +4207,15 @@
                 <c:pt idx="6" formatCode="0.00000">
                   <c:v>9.9143945152060597E-2</c:v>
                 </c:pt>
-                <c:pt idx="7" formatCode="0.00000">
-                  <c:v>-4.1760232547360499E-2</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>summer!$Y$26:$Y$36</c:f>
+              <c:f>summer!$Y$26:$Y$32</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0.19059894727801999</c:v>
                 </c:pt>
@@ -4236,9 +4236,6 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.49664162355941199</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>-0.27417249103342101</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4716,7 +4713,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:trendlineType val="linear"/>
+            <c:trendlineType val="log"/>
             <c:dispRSqr val="1"/>
             <c:dispEq val="0"/>
             <c:trendlineLbl>
@@ -4763,7 +4760,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>summer!$X$40:$X$50</c:f>
+              <c:f>summer!$X$38:$X$48</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="11"/>
@@ -4805,7 +4802,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>summer!$Y$40:$Y$50</c:f>
+              <c:f>summer!$Y$38:$Y$48</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="11"/>
@@ -5378,19 +5375,19 @@
                 <c:pt idx="2">
                   <c:v>0.21234239309632399</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="0.0000">
+                <c:pt idx="4" formatCode="0.0000">
                   <c:v>8.8732929175135894E-2</c:v>
                 </c:pt>
-                <c:pt idx="4" formatCode="0.0000">
+                <c:pt idx="5" formatCode="0.0000">
                   <c:v>0.10415722716452799</c:v>
                 </c:pt>
-                <c:pt idx="5" formatCode="0.0000">
+                <c:pt idx="6" formatCode="0.0000">
                   <c:v>4.66251429291673E-2</c:v>
                 </c:pt>
-                <c:pt idx="6" formatCode="0.0000">
+                <c:pt idx="7" formatCode="0.0000">
                   <c:v>9.0894558490112708E-3</c:v>
                 </c:pt>
-                <c:pt idx="7" formatCode="0.0000">
+                <c:pt idx="8" formatCode="0.0000">
                   <c:v>2.0373962034653699E-2</c:v>
                 </c:pt>
               </c:numCache>
@@ -5411,19 +5408,19 @@
                 <c:pt idx="2">
                   <c:v>77.803592516854394</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="General">
+                <c:pt idx="4" formatCode="General">
                   <c:v>113.72040256</c:v>
                 </c:pt>
-                <c:pt idx="4" formatCode="General">
+                <c:pt idx="5" formatCode="General">
                   <c:v>112.66319882000001</c:v>
                 </c:pt>
-                <c:pt idx="5" formatCode="General">
+                <c:pt idx="6" formatCode="General">
                   <c:v>114.89097618</c:v>
                 </c:pt>
-                <c:pt idx="6" formatCode="General">
+                <c:pt idx="7" formatCode="General">
                   <c:v>116.55531655999999</c:v>
                 </c:pt>
-                <c:pt idx="7" formatCode="General">
+                <c:pt idx="8" formatCode="General">
                   <c:v>115.75512236</c:v>
                 </c:pt>
               </c:numCache>
@@ -10412,13 +10409,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>463826</xdr:colOff>
+      <xdr:colOff>496956</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>99391</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>32</xdr:col>
-      <xdr:colOff>142553</xdr:colOff>
+      <xdr:colOff>175683</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>167746</xdr:rowOff>
     </xdr:to>
@@ -10487,16 +10484,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>38</xdr:col>
-      <xdr:colOff>157371</xdr:colOff>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>2</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>66261</xdr:rowOff>
+      <xdr:rowOff>57978</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>43</xdr:col>
-      <xdr:colOff>449010</xdr:colOff>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>291641</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>134616</xdr:rowOff>
+      <xdr:rowOff>126333</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -11824,6 +11821,9 @@
       <c r="W23" t="s">
         <v>83</v>
       </c>
+      <c r="AJ23" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="24" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -11872,7 +11872,7 @@
       <c r="X25" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="Y25" s="118" t="s">
+      <c r="Y25" s="106" t="s">
         <v>29</v>
       </c>
       <c r="AJ25" s="3" t="s">
@@ -11905,7 +11905,7 @@
       <c r="W26" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="X26" s="116">
+      <c r="X26" s="104">
         <v>8.8732929175135894E-2</v>
       </c>
       <c r="Y26" s="11">
@@ -11958,7 +11958,7 @@
       <c r="W27" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="X27" s="116">
+      <c r="X27" s="104">
         <v>0.10415722716452799</v>
       </c>
       <c r="Y27" s="11">
@@ -12011,61 +12011,55 @@
       <c r="W28" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="X28" s="116">
+      <c r="X28" s="104">
         <v>4.66251429291673E-2</v>
       </c>
       <c r="Y28" s="11">
         <v>0.40695810522245701</v>
       </c>
-      <c r="AJ28" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="AK28" s="117">
-        <v>8.8732929175135894E-2</v>
-      </c>
-      <c r="AL28" s="3">
-        <v>113.72040256</v>
-      </c>
+      <c r="AJ28" s="3"/>
+      <c r="AK28" s="6"/>
+      <c r="AL28" s="11"/>
     </row>
     <row r="29" spans="1:38" x14ac:dyDescent="0.25">
       <c r="H29" s="10"/>
       <c r="W29" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="X29" s="116">
+      <c r="X29" s="104">
         <v>9.0894558490112708E-3</v>
       </c>
       <c r="Y29" s="11">
         <v>5.4056282725128302E-2</v>
       </c>
       <c r="AJ29" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AK29" s="117">
-        <v>0.10415722716452799</v>
+        <v>76</v>
+      </c>
+      <c r="AK29" s="105">
+        <v>8.8732929175135894E-2</v>
       </c>
       <c r="AL29" s="3">
-        <v>112.66319882000001</v>
+        <v>113.72040256</v>
       </c>
     </row>
     <row r="30" spans="1:38" x14ac:dyDescent="0.25">
       <c r="W30" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="X30" s="116">
+      <c r="X30" s="104">
         <v>2.0373962034653699E-2</v>
       </c>
       <c r="Y30" s="11">
         <v>0.45125668170602201</v>
       </c>
       <c r="AJ30" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="AK30" s="117">
-        <v>4.66251429291673E-2</v>
+        <v>77</v>
+      </c>
+      <c r="AK30" s="105">
+        <v>0.10415722716452799</v>
       </c>
       <c r="AL30" s="3">
-        <v>114.89097618</v>
+        <v>112.66319882000001</v>
       </c>
     </row>
     <row r="31" spans="1:38" x14ac:dyDescent="0.25">
@@ -12079,13 +12073,13 @@
         <v>0.30708458237534503</v>
       </c>
       <c r="AJ31" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AK31" s="117">
-        <v>9.0894558490112708E-3</v>
+        <v>78</v>
+      </c>
+      <c r="AK31" s="105">
+        <v>4.66251429291673E-2</v>
       </c>
       <c r="AL31" s="3">
-        <v>116.55531655999999</v>
+        <v>114.89097618</v>
       </c>
     </row>
     <row r="32" spans="1:38" ht="27" x14ac:dyDescent="0.25">
@@ -12117,16 +12111,16 @@
         <v>0.49664162355941199</v>
       </c>
       <c r="AJ32" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AK32" s="117">
-        <v>2.0373962034653699E-2</v>
+        <v>79</v>
+      </c>
+      <c r="AK32" s="105">
+        <v>9.0894558490112708E-3</v>
       </c>
       <c r="AL32" s="3">
-        <v>115.75512236</v>
-      </c>
-    </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
+        <v>116.55531655999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>6</v>
       </c>
@@ -12137,17 +12131,17 @@
         <v>0.57681691180727601</v>
       </c>
       <c r="E33" s="10"/>
-      <c r="W33" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="X33" s="6">
-        <v>-4.1760232547360499E-2</v>
-      </c>
-      <c r="Y33" s="11">
-        <v>-0.27417249103342101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AJ33" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AK33" s="105">
+        <v>2.0373962034653699E-2</v>
+      </c>
+      <c r="AL33" s="3">
+        <v>115.75512236</v>
+      </c>
+    </row>
+    <row r="34" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>7</v>
       </c>
@@ -12158,11 +12152,8 @@
         <v>0.54443871754473905</v>
       </c>
       <c r="E34" s="3"/>
-      <c r="W34" s="3"/>
-      <c r="X34" s="6"/>
-      <c r="Y34" s="11"/>
-    </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>8</v>
       </c>
@@ -12185,7 +12176,7 @@
         <v>0.30708458237534503</v>
       </c>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>9</v>
       </c>
@@ -12208,7 +12199,7 @@
         <v>0.49664162355941199</v>
       </c>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>10</v>
       </c>
@@ -12230,8 +12221,11 @@
       <c r="G37" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W37" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>11</v>
       </c>
@@ -12253,8 +12247,17 @@
       <c r="G38" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W38" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="X38" s="104">
+        <v>6.8212961854365706E-2</v>
+      </c>
+      <c r="Y38" s="11">
+        <v>-0.14571780115724001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>15</v>
       </c>
@@ -12271,11 +12274,17 @@
       <c r="G39" s="11">
         <v>-0.27417249103342101</v>
       </c>
-      <c r="W39" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="W39" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="X39" s="104">
+        <v>4.9611646415268197E-2</v>
+      </c>
+      <c r="Y39" s="11">
+        <v>0.15611461722769501</v>
+      </c>
+    </row>
+    <row r="40" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>16</v>
       </c>
@@ -12298,28 +12307,28 @@
         <v>-0.27417249103342101</v>
       </c>
       <c r="W40" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="X40" s="116">
-        <v>6.8212961854365706E-2</v>
+        <v>75</v>
+      </c>
+      <c r="X40" s="104">
+        <v>0.107447815904682</v>
       </c>
       <c r="Y40" s="11">
-        <v>-0.14571780115724001</v>
-      </c>
-    </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.29322882322716898</v>
+      </c>
+    </row>
+    <row r="41" spans="1:38" x14ac:dyDescent="0.25">
       <c r="H41" s="10"/>
       <c r="W41" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="X41" s="116">
-        <v>4.9611646415268197E-2</v>
+        <v>77</v>
+      </c>
+      <c r="X41" s="104">
+        <v>9.9852529707758195E-2</v>
       </c>
       <c r="Y41" s="11">
-        <v>0.15611461722769501</v>
-      </c>
-    </row>
-    <row r="42" spans="1:25" ht="27" x14ac:dyDescent="0.25">
+        <v>0.499861288181496</v>
+      </c>
+    </row>
+    <row r="42" spans="1:38" ht="27" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="s">
         <v>33</v>
       </c>
@@ -12342,16 +12351,16 @@
         <v>70</v>
       </c>
       <c r="W42" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="X42" s="116">
-        <v>0.107447815904682</v>
+        <v>78</v>
+      </c>
+      <c r="X42" s="104">
+        <v>5.5815481283492403E-2</v>
       </c>
       <c r="Y42" s="11">
-        <v>0.29322882322716898</v>
-      </c>
-    </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.40695810522245701</v>
+      </c>
+    </row>
+    <row r="43" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>8</v>
       </c>
@@ -12377,16 +12386,16 @@
         <v>1.1737788669959504</v>
       </c>
       <c r="W43" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="X43" s="116">
-        <v>9.9852529707758195E-2</v>
+        <v>79</v>
+      </c>
+      <c r="X43" s="104">
+        <v>9.5391388976058394E-2</v>
       </c>
       <c r="Y43" s="11">
-        <v>0.499861288181496</v>
-      </c>
-    </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
+        <v>5.4056282725128302E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>9</v>
       </c>
@@ -12412,16 +12421,16 @@
         <v>1.0182769682576838</v>
       </c>
       <c r="W44" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="X44" s="116">
-        <v>5.5815481283492403E-2</v>
+        <v>80</v>
+      </c>
+      <c r="X44" s="104">
+        <v>0.115227328160236</v>
       </c>
       <c r="Y44" s="11">
-        <v>0.40695810522245701</v>
-      </c>
-    </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.26690920736687102</v>
+      </c>
+    </row>
+    <row r="45" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>10</v>
       </c>
@@ -12447,16 +12456,16 @@
         <v>1</v>
       </c>
       <c r="W45" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="X45" s="116">
-        <v>9.5391388976058394E-2</v>
+        <v>81</v>
+      </c>
+      <c r="X45" s="104">
+        <v>0.157732693122626</v>
       </c>
       <c r="Y45" s="11">
-        <v>5.4056282725128302E-2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.45125668170602201</v>
+      </c>
+    </row>
+    <row r="46" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>11</v>
       </c>
@@ -12482,16 +12491,16 @@
         <v>1</v>
       </c>
       <c r="W46" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="X46" s="116">
-        <v>0.115227328160236</v>
+        <v>82</v>
+      </c>
+      <c r="X46" s="104">
+        <v>0.121156039239802</v>
       </c>
       <c r="Y46" s="11">
-        <v>0.26690920736687102</v>
-      </c>
-    </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.51242235468873398</v>
+      </c>
+    </row>
+    <row r="47" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>16</v>
       </c>
@@ -12517,79 +12526,59 @@
         <v>1.045397189964473</v>
       </c>
       <c r="W47" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="X47" s="116">
-        <v>0.157732693122626</v>
+        <v>8</v>
+      </c>
+      <c r="X47" s="4">
+        <v>0.13984116014494999</v>
       </c>
       <c r="Y47" s="11">
-        <v>0.45125668170602201</v>
-      </c>
-    </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.30708458237534503</v>
+      </c>
+    </row>
+    <row r="48" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
       <c r="W48" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="X48" s="116">
-        <v>0.121156039239802</v>
+        <v>9</v>
+      </c>
+      <c r="X48" s="4">
+        <v>8.9326261366187695E-2</v>
       </c>
       <c r="Y48" s="11">
-        <v>0.51242235468873398</v>
-      </c>
-    </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.25">
+        <v>0.49664162355941199</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
-      <c r="W49" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="X49" s="4">
-        <v>0.13984116014494999</v>
-      </c>
-      <c r="Y49" s="11">
-        <v>0.30708458237534503</v>
-      </c>
-    </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="W50" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="X50" s="4">
-        <v>8.9326261366187695E-2</v>
-      </c>
-      <c r="Y50" s="11">
-        <v>0.49664162355941199</v>
-      </c>
-    </row>
-    <row r="51" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="106" t="s">
+    </row>
+    <row r="51" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="110" t="s">
         <v>58</v>
       </c>
-      <c r="B51" s="107"/>
-      <c r="C51" s="107"/>
-      <c r="D51" s="107"/>
-      <c r="E51" s="107"/>
-      <c r="F51" s="108"/>
+      <c r="B51" s="111"/>
+      <c r="C51" s="111"/>
+      <c r="D51" s="111"/>
+      <c r="E51" s="111"/>
+      <c r="F51" s="112"/>
       <c r="G51" s="30"/>
       <c r="H51" s="30"/>
       <c r="I51" s="31"/>
-      <c r="K51" s="106" t="s">
+      <c r="K51" s="110" t="s">
         <v>60</v>
       </c>
-      <c r="L51" s="107"/>
-      <c r="M51" s="107"/>
-      <c r="N51" s="107"/>
-      <c r="O51" s="107"/>
-      <c r="P51" s="108"/>
+      <c r="L51" s="111"/>
+      <c r="M51" s="111"/>
+      <c r="N51" s="111"/>
+      <c r="O51" s="111"/>
+      <c r="P51" s="112"/>
       <c r="Q51" s="30"/>
       <c r="R51" s="30"/>
       <c r="S51" s="31"/>
     </row>
-    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" s="45" t="s">
         <v>34</v>
       </c>
@@ -12612,11 +12601,8 @@
       <c r="Q52" s="34"/>
       <c r="R52" s="34"/>
       <c r="S52" s="35"/>
-      <c r="W52" s="3"/>
-      <c r="X52" s="4"/>
-      <c r="Y52" s="3"/>
-    </row>
-    <row r="53" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" s="36" t="s">
         <v>35</v>
       </c>
@@ -12644,7 +12630,7 @@
       <c r="R53" s="34"/>
       <c r="S53" s="35"/>
     </row>
-    <row r="54" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="36" t="s">
         <v>36</v>
       </c>
@@ -12672,7 +12658,7 @@
       <c r="R54" s="34"/>
       <c r="S54" s="35"/>
     </row>
-    <row r="55" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="36" t="s">
         <v>37</v>
       </c>
@@ -12700,10 +12686,8 @@
       <c r="R55" s="34"/>
       <c r="S55" s="35"/>
       <c r="V55" s="3"/>
-      <c r="W55" s="116"/>
-      <c r="X55" s="11"/>
-    </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" s="36" t="s">
         <v>38</v>
       </c>
@@ -12731,10 +12715,8 @@
       <c r="R56" s="34"/>
       <c r="S56" s="35"/>
       <c r="V56" s="3"/>
-      <c r="W56" s="116"/>
-      <c r="X56" s="11"/>
-    </row>
-    <row r="57" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="37" t="s">
         <v>39</v>
       </c>
@@ -12762,7 +12744,7 @@
       <c r="R57" s="34"/>
       <c r="S57" s="35"/>
     </row>
-    <row r="58" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A58" s="36"/>
       <c r="B58" s="34"/>
       <c r="C58" s="34"/>
@@ -12782,7 +12764,7 @@
       <c r="R58" s="34"/>
       <c r="S58" s="35"/>
     </row>
-    <row r="59" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="36" t="s">
         <v>40</v>
       </c>
@@ -12806,7 +12788,7 @@
       <c r="R59" s="34"/>
       <c r="S59" s="35"/>
     </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A60" s="39"/>
       <c r="B60" s="40" t="s">
         <v>45</v>
@@ -12846,7 +12828,7 @@
       <c r="R60" s="34"/>
       <c r="S60" s="35"/>
     </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A61" s="36" t="s">
         <v>41</v>
       </c>
@@ -12890,7 +12872,7 @@
       <c r="R61" s="34"/>
       <c r="S61" s="35"/>
     </row>
-    <row r="62" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A62" s="36" t="s">
         <v>42</v>
       </c>
@@ -12926,7 +12908,7 @@
       <c r="R62" s="34"/>
       <c r="S62" s="35"/>
     </row>
-    <row r="63" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="37" t="s">
         <v>43</v>
       </c>
@@ -12958,7 +12940,7 @@
       <c r="R63" s="34"/>
       <c r="S63" s="35"/>
     </row>
-    <row r="64" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="36"/>
       <c r="B64" s="34"/>
       <c r="C64" s="34"/>
@@ -13228,25 +13210,25 @@
       </c>
     </row>
     <row r="72" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="109" t="s">
+      <c r="A72" s="113" t="s">
         <v>59</v>
       </c>
-      <c r="B72" s="110"/>
-      <c r="C72" s="110"/>
-      <c r="D72" s="110"/>
-      <c r="E72" s="110"/>
-      <c r="F72" s="111"/>
+      <c r="B72" s="114"/>
+      <c r="C72" s="114"/>
+      <c r="D72" s="114"/>
+      <c r="E72" s="114"/>
+      <c r="F72" s="115"/>
       <c r="G72" s="47"/>
       <c r="H72" s="47"/>
       <c r="I72" s="48"/>
-      <c r="K72" s="109" t="s">
+      <c r="K72" s="113" t="s">
         <v>61</v>
       </c>
-      <c r="L72" s="110"/>
-      <c r="M72" s="110"/>
-      <c r="N72" s="110"/>
-      <c r="O72" s="110"/>
-      <c r="P72" s="111"/>
+      <c r="L72" s="114"/>
+      <c r="M72" s="114"/>
+      <c r="N72" s="114"/>
+      <c r="O72" s="114"/>
+      <c r="P72" s="115"/>
       <c r="Q72" s="47"/>
       <c r="R72" s="47"/>
       <c r="S72" s="48"/>
@@ -13881,25 +13863,25 @@
       </c>
     </row>
     <row r="92" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="112" t="s">
+      <c r="A92" s="116" t="s">
         <v>68</v>
       </c>
-      <c r="B92" s="113"/>
-      <c r="C92" s="113"/>
-      <c r="D92" s="113"/>
-      <c r="E92" s="113"/>
-      <c r="F92" s="114"/>
+      <c r="B92" s="117"/>
+      <c r="C92" s="117"/>
+      <c r="D92" s="117"/>
+      <c r="E92" s="117"/>
+      <c r="F92" s="118"/>
       <c r="G92" s="81"/>
       <c r="H92" s="81"/>
       <c r="I92" s="82"/>
-      <c r="K92" s="112" t="s">
+      <c r="K92" s="116" t="s">
         <v>69</v>
       </c>
-      <c r="L92" s="113"/>
-      <c r="M92" s="113"/>
-      <c r="N92" s="113"/>
-      <c r="O92" s="113"/>
-      <c r="P92" s="114"/>
+      <c r="L92" s="117"/>
+      <c r="M92" s="117"/>
+      <c r="N92" s="117"/>
+      <c r="O92" s="117"/>
+      <c r="P92" s="118"/>
       <c r="Q92" s="81"/>
       <c r="R92" s="81"/>
       <c r="S92" s="82"/>
@@ -14488,7 +14470,7 @@
       <c r="N109" s="79">
         <v>2.4820423187405729</v>
       </c>
-      <c r="O109" s="115">
+      <c r="O109" s="103">
         <v>0.13113982632319088</v>
       </c>
       <c r="P109" s="79">
@@ -14534,22 +14516,22 @@
       </c>
     </row>
     <row r="112" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A112" s="103" t="s">
+      <c r="A112" s="107" t="s">
         <v>66</v>
       </c>
-      <c r="B112" s="104"/>
-      <c r="C112" s="104"/>
-      <c r="D112" s="104"/>
-      <c r="E112" s="104"/>
-      <c r="F112" s="105"/>
-      <c r="K112" s="103" t="s">
+      <c r="B112" s="108"/>
+      <c r="C112" s="108"/>
+      <c r="D112" s="108"/>
+      <c r="E112" s="108"/>
+      <c r="F112" s="109"/>
+      <c r="K112" s="107" t="s">
         <v>67</v>
       </c>
-      <c r="L112" s="104"/>
-      <c r="M112" s="104"/>
-      <c r="N112" s="104"/>
-      <c r="O112" s="104"/>
-      <c r="P112" s="105"/>
+      <c r="L112" s="108"/>
+      <c r="M112" s="108"/>
+      <c r="N112" s="108"/>
+      <c r="O112" s="108"/>
+      <c r="P112" s="109"/>
     </row>
     <row r="113" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A113" s="87" t="s">
@@ -15331,25 +15313,25 @@
       <c r="T139" s="22"/>
     </row>
     <row r="140" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="106" t="s">
+      <c r="A140" s="110" t="s">
         <v>58</v>
       </c>
-      <c r="B140" s="107"/>
-      <c r="C140" s="107"/>
-      <c r="D140" s="107"/>
-      <c r="E140" s="107"/>
-      <c r="F140" s="108"/>
+      <c r="B140" s="111"/>
+      <c r="C140" s="111"/>
+      <c r="D140" s="111"/>
+      <c r="E140" s="111"/>
+      <c r="F140" s="112"/>
       <c r="G140" s="19"/>
       <c r="H140" s="19"/>
       <c r="I140" s="20"/>
-      <c r="K140" s="106" t="s">
+      <c r="K140" s="110" t="s">
         <v>60</v>
       </c>
-      <c r="L140" s="107"/>
-      <c r="M140" s="107"/>
-      <c r="N140" s="107"/>
-      <c r="O140" s="107"/>
-      <c r="P140" s="108"/>
+      <c r="L140" s="111"/>
+      <c r="M140" s="111"/>
+      <c r="N140" s="111"/>
+      <c r="O140" s="111"/>
+      <c r="P140" s="112"/>
       <c r="T140" s="22"/>
     </row>
     <row r="141" spans="1:20" x14ac:dyDescent="0.25">
@@ -15937,25 +15919,25 @@
       <c r="T159" s="22"/>
     </row>
     <row r="160" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="109" t="s">
+      <c r="A160" s="113" t="s">
         <v>59</v>
       </c>
-      <c r="B160" s="110"/>
-      <c r="C160" s="110"/>
-      <c r="D160" s="110"/>
-      <c r="E160" s="110"/>
-      <c r="F160" s="111"/>
+      <c r="B160" s="114"/>
+      <c r="C160" s="114"/>
+      <c r="D160" s="114"/>
+      <c r="E160" s="114"/>
+      <c r="F160" s="115"/>
       <c r="G160" s="19"/>
       <c r="H160" s="19"/>
       <c r="I160" s="20"/>
-      <c r="K160" s="109" t="s">
+      <c r="K160" s="113" t="s">
         <v>61</v>
       </c>
-      <c r="L160" s="110"/>
-      <c r="M160" s="110"/>
-      <c r="N160" s="110"/>
-      <c r="O160" s="110"/>
-      <c r="P160" s="111"/>
+      <c r="L160" s="114"/>
+      <c r="M160" s="114"/>
+      <c r="N160" s="114"/>
+      <c r="O160" s="114"/>
+      <c r="P160" s="115"/>
       <c r="T160" s="22"/>
     </row>
     <row r="161" spans="1:20" x14ac:dyDescent="0.25">
@@ -16543,25 +16525,25 @@
       <c r="T179" s="22"/>
     </row>
     <row r="180" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A180" s="112" t="s">
+      <c r="A180" s="116" t="s">
         <v>68</v>
       </c>
-      <c r="B180" s="113"/>
-      <c r="C180" s="113"/>
-      <c r="D180" s="113"/>
-      <c r="E180" s="113"/>
-      <c r="F180" s="114"/>
+      <c r="B180" s="117"/>
+      <c r="C180" s="117"/>
+      <c r="D180" s="117"/>
+      <c r="E180" s="117"/>
+      <c r="F180" s="118"/>
       <c r="G180" s="19"/>
       <c r="H180" s="19"/>
       <c r="I180" s="20"/>
-      <c r="K180" s="112" t="s">
+      <c r="K180" s="116" t="s">
         <v>69</v>
       </c>
-      <c r="L180" s="113"/>
-      <c r="M180" s="113"/>
-      <c r="N180" s="113"/>
-      <c r="O180" s="113"/>
-      <c r="P180" s="114"/>
+      <c r="L180" s="117"/>
+      <c r="M180" s="117"/>
+      <c r="N180" s="117"/>
+      <c r="O180" s="117"/>
+      <c r="P180" s="118"/>
       <c r="T180" s="22"/>
     </row>
     <row r="181" spans="1:20" x14ac:dyDescent="0.25">
@@ -17149,22 +17131,22 @@
       <c r="T199" s="22"/>
     </row>
     <row r="200" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="103" t="s">
+      <c r="A200" s="107" t="s">
         <v>66</v>
       </c>
-      <c r="B200" s="104"/>
-      <c r="C200" s="104"/>
-      <c r="D200" s="104"/>
-      <c r="E200" s="104"/>
-      <c r="F200" s="105"/>
-      <c r="K200" s="103" t="s">
+      <c r="B200" s="108"/>
+      <c r="C200" s="108"/>
+      <c r="D200" s="108"/>
+      <c r="E200" s="108"/>
+      <c r="F200" s="109"/>
+      <c r="K200" s="107" t="s">
         <v>67</v>
       </c>
-      <c r="L200" s="104"/>
-      <c r="M200" s="104"/>
-      <c r="N200" s="104"/>
-      <c r="O200" s="104"/>
-      <c r="P200" s="105"/>
+      <c r="L200" s="108"/>
+      <c r="M200" s="108"/>
+      <c r="N200" s="108"/>
+      <c r="O200" s="108"/>
+      <c r="P200" s="109"/>
       <c r="T200" s="22"/>
     </row>
     <row r="201" spans="1:20" x14ac:dyDescent="0.25">
@@ -17990,22 +17972,22 @@
       <c r="T229" s="22"/>
     </row>
     <row r="230" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A230" s="106" t="s">
+      <c r="A230" s="110" t="s">
         <v>58</v>
       </c>
-      <c r="B230" s="107"/>
-      <c r="C230" s="107"/>
-      <c r="D230" s="107"/>
-      <c r="E230" s="107"/>
-      <c r="F230" s="108"/>
-      <c r="K230" s="106" t="s">
+      <c r="B230" s="111"/>
+      <c r="C230" s="111"/>
+      <c r="D230" s="111"/>
+      <c r="E230" s="111"/>
+      <c r="F230" s="112"/>
+      <c r="K230" s="110" t="s">
         <v>60</v>
       </c>
-      <c r="L230" s="107"/>
-      <c r="M230" s="107"/>
-      <c r="N230" s="107"/>
-      <c r="O230" s="107"/>
-      <c r="P230" s="108"/>
+      <c r="L230" s="111"/>
+      <c r="M230" s="111"/>
+      <c r="N230" s="111"/>
+      <c r="O230" s="111"/>
+      <c r="P230" s="112"/>
       <c r="Q230" s="34"/>
       <c r="R230" s="34"/>
       <c r="S230" s="34"/>
@@ -18583,22 +18565,22 @@
       <c r="T249" s="22"/>
     </row>
     <row r="250" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A250" s="109" t="s">
+      <c r="A250" s="113" t="s">
         <v>59</v>
       </c>
-      <c r="B250" s="110"/>
-      <c r="C250" s="110"/>
-      <c r="D250" s="110"/>
-      <c r="E250" s="110"/>
-      <c r="F250" s="111"/>
-      <c r="K250" s="109" t="s">
+      <c r="B250" s="114"/>
+      <c r="C250" s="114"/>
+      <c r="D250" s="114"/>
+      <c r="E250" s="114"/>
+      <c r="F250" s="115"/>
+      <c r="K250" s="113" t="s">
         <v>61</v>
       </c>
-      <c r="L250" s="110"/>
-      <c r="M250" s="110"/>
-      <c r="N250" s="110"/>
-      <c r="O250" s="110"/>
-      <c r="P250" s="111"/>
+      <c r="L250" s="114"/>
+      <c r="M250" s="114"/>
+      <c r="N250" s="114"/>
+      <c r="O250" s="114"/>
+      <c r="P250" s="115"/>
       <c r="T250" s="22"/>
     </row>
     <row r="251" spans="1:20" x14ac:dyDescent="0.25">
@@ -19173,22 +19155,22 @@
       <c r="T269" s="22"/>
     </row>
     <row r="270" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A270" s="112" t="s">
+      <c r="A270" s="116" t="s">
         <v>59</v>
       </c>
-      <c r="B270" s="113"/>
-      <c r="C270" s="113"/>
-      <c r="D270" s="113"/>
-      <c r="E270" s="113"/>
-      <c r="F270" s="114"/>
-      <c r="K270" s="112" t="s">
+      <c r="B270" s="117"/>
+      <c r="C270" s="117"/>
+      <c r="D270" s="117"/>
+      <c r="E270" s="117"/>
+      <c r="F270" s="118"/>
+      <c r="K270" s="116" t="s">
         <v>61</v>
       </c>
-      <c r="L270" s="113"/>
-      <c r="M270" s="113"/>
-      <c r="N270" s="113"/>
-      <c r="O270" s="113"/>
-      <c r="P270" s="114"/>
+      <c r="L270" s="117"/>
+      <c r="M270" s="117"/>
+      <c r="N270" s="117"/>
+      <c r="O270" s="117"/>
+      <c r="P270" s="118"/>
       <c r="T270" s="22"/>
     </row>
     <row r="271" spans="1:20" x14ac:dyDescent="0.25">
@@ -19763,22 +19745,22 @@
       <c r="T289" s="22"/>
     </row>
     <row r="290" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A290" s="103" t="s">
+      <c r="A290" s="107" t="s">
         <v>66</v>
       </c>
-      <c r="B290" s="104"/>
-      <c r="C290" s="104"/>
-      <c r="D290" s="104"/>
-      <c r="E290" s="104"/>
-      <c r="F290" s="105"/>
-      <c r="K290" s="103" t="s">
+      <c r="B290" s="108"/>
+      <c r="C290" s="108"/>
+      <c r="D290" s="108"/>
+      <c r="E290" s="108"/>
+      <c r="F290" s="109"/>
+      <c r="K290" s="107" t="s">
         <v>67</v>
       </c>
-      <c r="L290" s="104"/>
-      <c r="M290" s="104"/>
-      <c r="N290" s="104"/>
-      <c r="O290" s="104"/>
-      <c r="P290" s="105"/>
+      <c r="L290" s="108"/>
+      <c r="M290" s="108"/>
+      <c r="N290" s="108"/>
+      <c r="O290" s="108"/>
+      <c r="P290" s="109"/>
       <c r="T290" s="22"/>
     </row>
     <row r="291" spans="1:20" x14ac:dyDescent="0.25">
@@ -20440,18 +20422,16 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="K250:P250"/>
-    <mergeCell ref="K270:P270"/>
+    <mergeCell ref="A112:F112"/>
+    <mergeCell ref="K112:P112"/>
+    <mergeCell ref="A200:F200"/>
+    <mergeCell ref="K200:P200"/>
     <mergeCell ref="A51:F51"/>
     <mergeCell ref="A72:F72"/>
     <mergeCell ref="K51:P51"/>
     <mergeCell ref="K72:P72"/>
     <mergeCell ref="A92:F92"/>
     <mergeCell ref="K92:P92"/>
-    <mergeCell ref="A112:F112"/>
-    <mergeCell ref="K112:P112"/>
-    <mergeCell ref="A200:F200"/>
-    <mergeCell ref="K200:P200"/>
     <mergeCell ref="A290:F290"/>
     <mergeCell ref="K290:P290"/>
     <mergeCell ref="A140:F140"/>
@@ -20464,6 +20444,8 @@
     <mergeCell ref="A250:F250"/>
     <mergeCell ref="A270:F270"/>
     <mergeCell ref="K230:P230"/>
+    <mergeCell ref="K250:P250"/>
+    <mergeCell ref="K270:P270"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>